<commit_message>
Complete MSW 21-day field report with locked photos, 24/04 Jal Ganga entry, and documentation
</commit_message>
<xml_diff>
--- a/gudiya-Mausi-MSW-work/परामर्शदाता_व्यावहारिक_कार्य_प्रतिवेदन_स्नेहलता_मिश्रा.xlsx
+++ b/gudiya-Mausi-MSW-work/परामर्शदाता_व्यावहारिक_कार्य_प्रतिवेदन_स्नेहलता_मिश्रा.xlsx
@@ -528,6 +528,33 @@
   <oneCellAnchor>
     <from>
       <col>6</col>
+      <colOff>509587</colOff>
+      <row>15</row>
+      <rowOff>111125</rowOff>
+    </from>
+    <ext cx="895350" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Photo 13" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noMove="1" noResize="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
       <colOff>671512</colOff>
       <row>16</row>
       <rowOff>111125</rowOff>
@@ -541,7 +568,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
+        <a:blip cstate="print" r:embed="rId14"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -568,7 +595,34 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>385762</colOff>
+      <row>18</row>
+      <rowOff>111125</rowOff>
+    </from>
+    <ext cx="1143000" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Photo 16" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noMove="1" noResize="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -583,19 +637,19 @@
     <from>
       <col>6</col>
       <colOff>195262</colOff>
-      <row>18</row>
+      <row>19</row>
       <rowOff>377825</rowOff>
     </from>
     <ext cx="1524000" cy="704850"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="16" name="Photo 16" descr="Picture"/>
-        <cNvPicPr>
-          <a:picLocks noMove="1" noResize="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
+        <cNvPr id="17" name="Photo 17" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noMove="1" noResize="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -610,37 +664,10 @@
     <from>
       <col>6</col>
       <colOff>319087</colOff>
-      <row>19</row>
-      <rowOff>111125</rowOff>
-    </from>
-    <ext cx="1276350" cy="1238250"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="17" name="Photo 17" descr="Picture"/>
-        <cNvPicPr>
-          <a:picLocks noMove="1" noResize="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>447675</colOff>
       <row>20</row>
       <rowOff>111125</rowOff>
     </from>
-    <ext cx="1019175" cy="1238250"/>
+    <ext cx="1276350" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="18" name="Photo 18" descr="Picture"/>
@@ -649,34 +676,61 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>476250</colOff>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>447675</colOff>
       <row>21</row>
       <rowOff>111125</rowOff>
     </from>
+    <ext cx="1019175" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Photo 19" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noMove="1" noResize="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>476250</colOff>
+      <row>22</row>
+      <rowOff>111125</rowOff>
+    </from>
     <ext cx="962025" cy="1238250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="19" name="Photo 19" descr="Picture"/>
-        <cNvPicPr>
-          <a:picLocks noMove="1" noResize="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
+        <cNvPr id="20" name="Photo 20" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noMove="1" noResize="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -691,19 +745,19 @@
     <from>
       <col>6</col>
       <colOff>195262</colOff>
-      <row>22</row>
+      <row>23</row>
       <rowOff>373062</rowOff>
     </from>
     <ext cx="1524000" cy="714375"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="20" name="Photo 20" descr="Picture"/>
-        <cNvPicPr>
-          <a:picLocks noMove="1" noResize="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
+        <cNvPr id="21" name="Photo 21" descr="Picture"/>
+        <cNvPicPr>
+          <a:picLocks noMove="1" noResize="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1006,7 +1060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1221,7 +1275,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>25/03/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1500,12 +1554,12 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>रसेना</t>
+          <t>महाराजपुर</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1531,7 +1585,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1562,17 +1616,17 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>डोभी</t>
+          <t>महाराजपुर</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>महिलाओं के साथ भजन-पूजन कार्य</t>
+          <t>जल गंगा संवर्धन अभियान - जल संरक्षण पे दीवार लेखन</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr"/>
@@ -1593,17 +1647,17 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>महाराजपुर</t>
+          <t>डोभी</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>छात्र-छात्राओं के साथ सेक्टर भ्रमण</t>
+          <t>महिलाओं के साथ भजन-पूजन कार्य</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr"/>
@@ -1624,17 +1678,17 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>सिमरिया</t>
+          <t>महाराजपुर</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>MSW छात्रा से सम्पर्क</t>
+          <t>छात्र-छात्राओं के साथ सेक्टर भ्रमण</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr"/>
@@ -1655,17 +1709,17 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>डोभी</t>
+          <t>सिमरिया</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>महिलाओं के साथ बैठक एवं पर्यावरण / जल संवर्धन अभियान चर्चा</t>
+          <t>MSW छात्रा से सम्पर्क</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
@@ -1686,20 +1740,51 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
+          <t>29/04/2026</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>डोभी</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>महिलाओं के साथ बैठक एवं पर्यावरण / जल संवर्धन अभियान चर्चा</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24" ht="115" customHeight="1">
+      <c r="A24" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>सागर</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>देवरी</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
           <t>30/04/2026</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>रीछई</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>छात्र-छात्राओं से संपर्क एवं असाइनमेंट कार्य चर्चा</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>